<commit_message>
AI Course Builder: attach YouTube videos to generated sessions
The AI writes a search phrase per session; the server searches the
YouTube Data API v3 (embeddable, public, safe search, 2 min to 3 h,
not live), caches results 12 h and searches each phrase once. The
review step finds videos automatically with Another / Remove / Paste
link, never repeats a video within a course, and saves videoUrl,
videoTitle and videoChannel on each session. Course Builder > Content
gains "Find YouTube videos" for existing courses. The key is set in
Settings > Integrations > YouTube videos (or YOUTUBE_API_KEY) and never
leaves the server. Adds tests/videos.test.js, gateway permission
scenarios, docs and manual cases CB-21..CB-30.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/SDC-Learn-Manual-Test-Suite-Full.xlsx
+++ b/docs/testing/SDC-Learn-Manual-Test-Suite-Full.xlsx
@@ -1889,7 +1889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2973,8 +2973,518 @@
       <c r="L22" s="8" t="inlineStr"/>
       <c r="M22" s="8" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>CB-21</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>YouTube key in Integrations</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>A YouTube Data API v3 key (enter it yourself)</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Settings → Integrations → YouTube videos: paste key, Save key, Test; then try a wrong key</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Configured, key masked; Test finds videos; a wrong key gives "YouTube refused the API key"</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr"/>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr"/>
+      <c r="L23" s="8" t="inlineStr"/>
+      <c r="M23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>CB-22</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Videos found automatically</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>YouTube key saved; AI provider configured</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Generate an outline → Review</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>"Finding a video for each session…", then each session shows a thumbnail, title, channel and length; "N of M sessions" count</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr"/>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr"/>
+      <c r="L24" s="8" t="inlineStr"/>
+      <c r="M24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>CB-23</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>No repeated videos</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Review step with videos</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Compare the videos of all sessions</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>No video appears in two sessions of the course</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr"/>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr"/>
+      <c r="L25" s="8" t="inlineStr"/>
+      <c r="M25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>CB-24</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Another / Remove / Paste link</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Review step with videos</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Another video on one session; Remove on another; Paste a YouTube link (try a non-YouTube link first)</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Video swaps; removed shows "No video"; non-YouTube link refused; pasted video shown</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr"/>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr"/>
+      <c r="L26" s="8" t="inlineStr"/>
+      <c r="M26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>CB-25</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Find videos again</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Some sessions without a video</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Find videos for sessions without one</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>Only empty sessions are searched; others keep their video</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr"/>
+      <c r="L27" s="8" t="inlineStr"/>
+      <c r="M27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>CB-26</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Videos saved with the draft</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Review with videos</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Create draft course → Sessions tab → open a session as learner preview</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Sessions list shows "video"; session page plays the YouTube video with its title and channel under it</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr"/>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K28" s="8" t="inlineStr"/>
+      <c r="L28" s="8" t="inlineStr"/>
+      <c r="M28" s="8" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>CB-27</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>No YouTube key</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>No YouTube key set</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Generate an outline → Review</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Clear note that no key is set; draft can still be created without videos</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr"/>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K29" s="8" t="inlineStr"/>
+      <c r="L29" s="8" t="inlineStr"/>
+      <c r="M29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>CB-28</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Find videos for an existing course</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>A course with sessions that have no video</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Course Builder → Content → Find YouTube videos (N) → confirm</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Videos attached to empty sessions only; existing videos/recordings unchanged</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr"/>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K30" s="8" t="inlineStr"/>
+      <c r="L30" s="8" t="inlineStr"/>
+      <c r="M30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>CB-29</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Changing a found video</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>admin@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>A session with a found video</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Sessions tab → edit the session → change the video URL → save</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>New video plays; the old title/channel line is gone</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr"/>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K31" s="8" t="inlineStr"/>
+      <c r="L31" s="8" t="inlineStr"/>
+      <c r="M31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>CB-30</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>AI Course Builder</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Who can search videos</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>instructor@sdclearn.demo</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Feature on</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>As learner / instructor without course create, try the generator</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>No access; only course creators (and editors in the Content tab) can search</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr"/>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="K32" s="8" t="inlineStr"/>
+      <c r="L32" s="8" t="inlineStr"/>
+      <c r="M32" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="J3:J22">
+  <conditionalFormatting sqref="J3:J32">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2989,7 +3499,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J3:J22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3:J32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4383,26 +4893,26 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C12">
-        <f>COUNTIF('10 AI Course Builder'!J3:J22,"Pass")</f>
+        <f>COUNTIF('10 AI Course Builder'!J3:J32,"Pass")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>COUNTIF('10 AI Course Builder'!J3:J22,"Fail")</f>
+        <f>COUNTIF('10 AI Course Builder'!J3:J32,"Fail")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>COUNTIF('10 AI Course Builder'!J3:J22,"Blocked")</f>
+        <f>COUNTIF('10 AI Course Builder'!J3:J32,"Blocked")</f>
         <v/>
       </c>
       <c r="F12">
-        <f>COUNTIF('10 AI Course Builder'!J3:J22,"N/A")</f>
+        <f>COUNTIF('10 AI Course Builder'!J3:J32,"N/A")</f>
         <v/>
       </c>
       <c r="G12">
-        <f>COUNTIF('10 AI Course Builder'!J3:J22,"Not Run")</f>
+        <f>COUNTIF('10 AI Course Builder'!J3:J32,"Not Run")</f>
         <v/>
       </c>
       <c r="H12" s="5">

</xml_diff>